<commit_message>
feat: most of fact done
</commit_message>
<xml_diff>
--- a/project/stage02/data/circuits.xlsx
+++ b/project/stage02/data/circuits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jantar\uni-data-warehouse\project\stage02\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721E2372-9CBE-4680-A2CE-4CC0EF8DCEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C179E3-0D65-4C7E-ADF0-EE6DD79F78BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1432,6 +1432,7 @@
   <dimension ref="A1:I78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="67.7109375" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>